<commit_message>
system prompt and research goal
</commit_message>
<xml_diff>
--- a/gantt.xlsx
+++ b/gantt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mikolajmazur/Documents/studia/inz/llm-persona-evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A32B2E-F077-6947-A1B5-46EE5538E2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A3F22A3-EADD-ED45-86AA-1962CC9F74B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3760" yWindow="-20540" windowWidth="30240" windowHeight="17360" xr2:uid="{07D868FB-0D69-C04A-95E7-840297A8853B}"/>
+    <workbookView xWindow="10640" yWindow="-20400" windowWidth="30240" windowHeight="17360" xr2:uid="{07D868FB-0D69-C04A-95E7-840297A8853B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -163,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
@@ -175,6 +175,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -571,7 +572,7 @@
       <c r="A6" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="3"/>
+      <c r="B6" s="6"/>
       <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -587,7 +588,7 @@
       <c r="A9" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="5"/>
+      <c r="C9" s="7"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">

</xml_diff>

<commit_message>
readme update - more details added
</commit_message>
<xml_diff>
--- a/gantt.xlsx
+++ b/gantt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mikolajmazur/Documents/studia/inz/llm-persona-evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A3F22A3-EADD-ED45-86AA-1962CC9F74B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CE2AF6-A941-D94D-9EBB-199E2F50A918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10640" yWindow="-20400" windowWidth="30240" windowHeight="17360" xr2:uid="{07D868FB-0D69-C04A-95E7-840297A8853B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>opensource models selection</t>
   </si>
@@ -87,9 +87,6 @@
   </si>
   <si>
     <t>judging results</t>
-  </si>
-  <si>
-    <t>aggregsating results</t>
   </si>
   <si>
     <t>project delivery</t>
@@ -640,7 +637,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
@@ -685,7 +682,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I25" s="5"/>
     </row>

</xml_diff>

<commit_message>
repo and plan refactor
</commit_message>
<xml_diff>
--- a/gantt.xlsx
+++ b/gantt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mikolajmazur/Documents/studia/inz/llm-persona-evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CE2AF6-A941-D94D-9EBB-199E2F50A918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEFE574B-CCA1-FC46-B74E-A212EAA424E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10640" yWindow="-20400" windowWidth="30240" windowHeight="17360" xr2:uid="{07D868FB-0D69-C04A-95E7-840297A8853B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" xr2:uid="{07D868FB-0D69-C04A-95E7-840297A8853B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>opensource models selection</t>
   </si>
@@ -53,9 +53,6 @@
     <t>basic steps</t>
   </si>
   <si>
-    <t>script for hpc testing</t>
-  </si>
-  <si>
     <t>system prompt</t>
   </si>
   <si>
@@ -90,13 +87,19 @@
   </si>
   <si>
     <t>project delivery</t>
+  </si>
+  <si>
+    <t>script for testing demo</t>
+  </si>
+  <si>
+    <t>script for target testing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -118,8 +121,15 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -136,6 +146,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1A983"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -160,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
@@ -173,6 +189,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,13 +527,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33CE6878-6A04-CD49-B40D-9FCEF3E2A9C6}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="5.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="1">
         <v>46104</v>
       </c>
@@ -530,161 +551,261 @@
         <v>46132</v>
       </c>
       <c r="G1" s="1">
+        <v>46132</v>
+      </c>
+      <c r="H1" s="1">
         <v>46139</v>
       </c>
-      <c r="H1" s="1">
+      <c r="I1" s="1">
         <v>46146</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>46147</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="4"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="4"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="4"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C7" s="4"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="4"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="C9" s="7"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="10"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="9"/>
+      <c r="E11" s="5"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="9"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="9"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="3"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="C14" s="9"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="7"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="E16" s="5"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="11"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="4"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C13" s="4"/>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="3"/>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="G19" s="9"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="3"/>
-      <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="3"/>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>12</v>
-      </c>
-      <c r="G21" s="5"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>14</v>
-      </c>
-      <c r="H22" s="3"/>
-      <c r="I22" s="4"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="9"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>13</v>
       </c>
-      <c r="H23" s="3"/>
-      <c r="I23" s="4"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I24" s="4"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>17</v>
-      </c>
-      <c r="I25" s="5"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="9"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="9"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="9"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="9"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
evaluation script ready for testing
</commit_message>
<xml_diff>
--- a/gantt.xlsx
+++ b/gantt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mikolajmazur/Documents/studia/inz/llm-persona-evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEFE574B-CCA1-FC46-B74E-A212EAA424E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD4D1C61-A348-B342-A731-02D53BA2DF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" xr2:uid="{07D868FB-0D69-C04A-95E7-840297A8853B}"/>
   </bookViews>
@@ -129,18 +129,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -150,7 +144,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1A983"/>
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -176,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
@@ -184,15 +178,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -527,14 +516,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33CE6878-6A04-CD49-B40D-9FCEF3E2A9C6}">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="5.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="1">
         <v>46104</v>
       </c>
@@ -563,249 +552,152 @@
         <v>46147</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="4"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B3" s="4"/>
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="4"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B4" s="4"/>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="4"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B5" s="4"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C7" s="4"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B6" s="4"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="4"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="7"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="C9" s="5"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="10"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="9"/>
       <c r="E11" s="5"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E12" s="3"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="3"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C14" s="9"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E13" s="3"/>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="9"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>7</v>
       </c>
       <c r="E16" s="5"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>9</v>
       </c>
-      <c r="F17" s="3"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="F17" s="4"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>14</v>
       </c>
-      <c r="G18" s="11"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>15</v>
       </c>
-      <c r="G19" s="9"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="H19" s="4"/>
+      <c r="I19" s="3"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="I20" s="3"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I21" s="3"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
       <c r="I22" s="5"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J22" s="3"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
       <c r="I23" s="5"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="9"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J23" s="3"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>12</v>
       </c>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
       <c r="I24" s="5"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="9"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="9"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J24" s="3"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J25" s="3"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>16</v>
       </c>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
       <c r="J26" s="5"/>
-      <c r="K26" s="9"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="9"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="9"/>
-      <c r="K29" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>